<commit_message>
12/18/2025 Update: New perinatal conditions added to CCB Condition List
</commit_message>
<xml_diff>
--- a/Partner Resources/ICD10 to CCB Causes/death.File.Vars.xlsx
+++ b/Partner Resources/ICD10 to CCB Causes/death.File.Vars.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\FusionData\0.CCB\Partner Resources\ICD10 to CCB Causes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4AB031D-18E0-4386-8E0D-F38C82F37ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB0C368C-6D71-4DFE-9D39-9A329986977B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2940" yWindow="870" windowWidth="33945" windowHeight="18090" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="variableNames" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>F19</t>
   </si>
@@ -72,6 +72,12 @@
   </si>
   <si>
     <t>F1</t>
+  </si>
+  <si>
+    <t>age</t>
+  </si>
+  <si>
+    <t>F12</t>
   </si>
 </sst>
 </file>
@@ -113,12 +119,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -401,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="28.85546875" bestFit="1" customWidth="1"/>
@@ -425,33 +434,41 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>1</v>
+        <v>12</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B7" s="1" t="s">
         <v>2</v>
       </c>
     </row>

</xml_diff>